<commit_message>
add more us etfs
</commit_message>
<xml_diff>
--- a/final_result/etf/momentum_us_etfs.xlsx
+++ b/final_result/etf/momentum_us_etfs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,42 +429,37 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>9EMA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Close_Below_9EMA</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Return_1W</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Return_2W</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Return_1M</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Return_3M</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Rank_2W</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Rank_1M</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Rank_3M</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Final_Rank</t>
         </is>
       </c>
     </row>
@@ -474,32 +469,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>WGMI</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-1.7</v>
+        <v>65.86</v>
       </c>
       <c r="D2" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.1</v>
+        <v>66.45</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F2" t="n">
-        <v>44.3</v>
+        <v>-6.9</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>6.3</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>13.5</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J2" t="n">
-        <v>2</v>
+        <v>76.40000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -508,32 +502,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EWY</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-5.6</v>
+        <v>571.23</v>
       </c>
       <c r="D3" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="E3" t="n">
-        <v>17.8</v>
+        <v>571.21</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
       </c>
       <c r="F3" t="n">
-        <v>34</v>
+        <v>-0.1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>6.3</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J3" t="n">
-        <v>2.600000000000001</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -542,32 +535,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>SOXQ</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9.699999999999999</v>
+        <v>101.47</v>
       </c>
       <c r="D4" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>26.3</v>
+        <v>101.71</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F4" t="n">
-        <v>92.2</v>
+        <v>-0.5</v>
       </c>
       <c r="G4" t="n">
-        <v>13</v>
+        <v>5.6</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>9.5</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3.4</v>
+        <v>65.2</v>
       </c>
     </row>
     <row r="5">
@@ -576,32 +568,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>CHPS</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7</v>
+        <v>90.47</v>
       </c>
       <c r="D5" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="E5" t="n">
-        <v>14.5</v>
+        <v>91.25</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F5" t="n">
-        <v>26.8</v>
+        <v>-2</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>5.3</v>
       </c>
       <c r="H5" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
-      </c>
-      <c r="J5" t="n">
-        <v>4.6</v>
+        <v>65.5</v>
       </c>
     </row>
     <row r="6">
@@ -610,32 +601,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TAN</t>
+          <t>ARTY</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>73.94</v>
       </c>
       <c r="D6" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="E6" t="n">
-        <v>15.8</v>
+        <v>74.48999999999999</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F6" t="n">
-        <v>10.2</v>
+        <v>-5.3</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>8.1</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
-      </c>
-      <c r="J6" t="n">
-        <v>7.200000000000001</v>
+        <v>50.2</v>
       </c>
     </row>
     <row r="7">
@@ -644,32 +634,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ICLN</t>
+          <t>FTXL</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>258</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>11.2</v>
+        <v>259.53</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F7" t="n">
-        <v>17.2</v>
+        <v>-0.4</v>
       </c>
       <c r="G7" t="n">
-        <v>10</v>
+        <v>4.1</v>
       </c>
       <c r="H7" t="n">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="I7" t="n">
-        <v>9</v>
-      </c>
-      <c r="J7" t="n">
-        <v>8</v>
+        <v>73.8</v>
       </c>
     </row>
     <row r="8">
@@ -678,32 +667,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>CHAT</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-0.1</v>
+        <v>93.56999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="E8" t="n">
-        <v>9.5</v>
+        <v>95.92</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F8" t="n">
-        <v>18.2</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>5.5</v>
+        <v>4.2</v>
       </c>
       <c r="H8" t="n">
-        <v>9.5</v>
+        <v>8.6</v>
       </c>
       <c r="I8" t="n">
-        <v>8</v>
-      </c>
-      <c r="J8" t="n">
-        <v>8.100000000000001</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="9">
@@ -712,32 +700,31 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DBC</t>
+          <t>XNTK</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.7</v>
+        <v>365.48</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>10</v>
+        <v>367.7</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F9" t="n">
-        <v>30.4</v>
+        <v>-3.1</v>
       </c>
       <c r="G9" t="n">
-        <v>19</v>
+        <v>4.8</v>
       </c>
       <c r="H9" t="n">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" t="n">
-        <v>8.4</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="10">
@@ -746,32 +733,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EWT</t>
+          <t>WTAI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-4.8</v>
+        <v>43.3</v>
       </c>
       <c r="D10" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="E10" t="n">
-        <v>10</v>
+        <v>43.97</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F10" t="n">
-        <v>25.3</v>
+        <v>-5.6</v>
       </c>
       <c r="G10" t="n">
-        <v>15.5</v>
+        <v>4</v>
       </c>
       <c r="H10" t="n">
-        <v>7.5</v>
+        <v>6.4</v>
       </c>
       <c r="I10" t="n">
-        <v>6</v>
-      </c>
-      <c r="J10" t="n">
-        <v>8.5</v>
+        <v>47.7</v>
       </c>
     </row>
     <row r="11">
@@ -780,32 +766,31 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MTUM</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.9</v>
+        <v>597.65</v>
       </c>
       <c r="D11" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="E11" t="n">
-        <v>8.9</v>
+        <v>600.84</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
       </c>
       <c r="F11" t="n">
-        <v>19</v>
+        <v>-1.7</v>
       </c>
       <c r="G11" t="n">
-        <v>7</v>
+        <v>3.7</v>
       </c>
       <c r="H11" t="n">
-        <v>11</v>
+        <v>5.5</v>
       </c>
       <c r="I11" t="n">
-        <v>7</v>
-      </c>
-      <c r="J11" t="n">
-        <v>8.600000000000001</v>
+        <v>51.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>